<commit_message>
Restore user's version of IT23861718_Assignment1.xlsx
</commit_message>
<xml_diff>
--- a/IT23861718_Assignment1.xlsx
+++ b/IT23861718_Assignment1.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -55,6 +55,12 @@
       <color theme="1"/>
       <sz val="8"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <sz val="8"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -70,7 +76,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -93,11 +99,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -117,6 +138,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -483,8 +510,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H51"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <dimension ref="A1:H52"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4" outlineLevelCol="0"/>
   <cols>
     <col width="10.88671875" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
@@ -557,7 +584,11 @@
           <t>නිමල් ඔයාට සැප සනීප කොහොමද?</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr"/>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>නිමල් ඔයාට සාප සනීප කොහොමද?</t>
+        </is>
+      </c>
       <c r="F2" s="6" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -568,9 +599,9 @@
           <t>Question forms</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>Evidence: 'sapa' is incorrectly output as 'සපා' instead of correct 'සැප' — the 'æ' vowel (ැ) is missing, changing the word meaning. Comma after name 'supun' is also dropped.</t>
+      <c r="H2" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: 'sapa' is incorrectly output as 'සාප' instead of correct 'සැප' — the 'æ' vowel (ැ) is missing, changing the word from 'healthy/well' to a curse word. The comma after person name 'nimal' is also dropped in the output.</t>
         </is>
       </c>
     </row>
@@ -595,10 +626,14 @@
           <t>ඔයාට කොහොමද එදාට එන්න පුලුවන්ද?</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>ඔයාට කොහොමද එදාට එන්න පුළුවන්ද?</t>
+        </is>
+      </c>
       <c r="F3" s="6" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -606,9 +641,9 @@
           <t>Question forms</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>Evidence: 'puluwnda' is output as 'පුළුවන්ද' using the retroflex 'ළ' instead of plain 'ල' — spelling variant with missing vowel produces a different character in Sinhala output.</t>
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: 'puluwnda' is output as 'පුළුවන්ද' using the retroflex letter 'ළ' instead of plain 'ල' as in expected 'පුලුවන්ද' — the abbreviated spelling variant with missing vowel 'a' causes the system to apply a different Sinhala character.</t>
         </is>
       </c>
     </row>
@@ -640,7 +675,7 @@
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -648,9 +683,9 @@
           <t>Command forms</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>Evidence: The system fails to maintain English technical terms such as 'print' and 'urgent' in their original form. Instead, it attempts to transliterate them phonetically into Sinhala (e.g., 'ප්‍රින්ට්'), which deviates from the expected output.</t>
+      <c r="H4" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: English technical term 'print' is phonetically converted to 'ප්රින්ට්' instead of being preserved in its original English form as required in the expected output — system applies Sinhala phonetics to English words that should remain unchanged.</t>
         </is>
       </c>
     </row>
@@ -662,23 +697,27 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>macho server ekata log wela database eka balanna. eke security update ekak daddi backup ekak ganna mathaka thiyaganna. server eka restart karanna epa thama. meka urgent case ekak nisa ikmanata iwara karala mata email ekak danna. oya meka iwara karala mtkwa mcn msg ekak danna</t>
+          <t>mchn me msg eka English walin thiyala 'ASAP' kalla Capital danna, ethakota 'urgent' kalla bold krla denda puluwanda</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>"මචෝ server එකට log වෙලා database එක බලන්න. ඒකේ security update එකක් දද්දී backup එකක් ගන්න මතක තියාගන්න. server එක restart කරන්න එපා තාම. මේක urgent case එකක් නිසා ඉක්මනට ඉවර කරලා මට email එකක් දාන්න. ඔයා මේක ඉවර කරලා මතක ඇතුව මචං msg එකක් දාන්න</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr"/>
+          <t>මචං මේ msg එක English වලින් තියලා 'ASAP' කෑල්ල Capital දාන්න, එතකොට 'urgent' කෑල්ල bold කරලා දෙන්න පුළුවන්ද</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>මචන් මේ msg එක English වලින් තියලා 'ASAP' කල්ල Capital දාන්න, එතකොට 'උර්ගෙන්ට්' කාලය බෝල්ඩ් කරලා දෙන්ඩ පුලුවන්ද</t>
+        </is>
+      </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -686,9 +725,9 @@
           <t>Command forms</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>Evidence: In a long command containing multiple technical terms ('server', 'database', 'backup', 'security'), the system incorrectly converts all English terms into phonetic Sinhala. Additionally, it fails to recognize the slang 'mcn' and the shortened word 'mtkwa', leading to significant transliteration errors.</t>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: Multiple English terms in the command ('mchn', 'msg', 'ASAP', 'Capital', 'bold') are either phonetically converted to incorrect Sinhala or produce garbled output — 'mchn' becomes 'ම්ච්න්', 'urgent' becomes 'උර්ගෙන්ට්', demonstrating the system fails to handle abbreviated Singlish commands with mixed English content.</t>
         </is>
       </c>
     </row>
@@ -713,10 +752,14 @@
           <t>සුබ පැතුම්! දැන්  ඔයාට ගෙදරක් තියනවා</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>සුබ පතුම්!දැන් ඔයාට ගෙදරක් තියනවා</t>
+        </is>
+      </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -724,9 +767,9 @@
           <t>Greetings</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>Evidence: 'siye' output as 'සියේ' instead of 'සීයෙ' — wrong vowel length. 'pathum' becomes 'පතුම්' instead of 'පැතුම්' — missing 'æ' vowel (ැ). Space after '!' also dropped.</t>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: 'pathum' is output as 'පතුම්' instead of correct 'පැතුම්' — the 'æ' vowel (ැ) is missing, changing the meaning. Space after '!' is also dropped causing '!දැන්' to be joined without space.</t>
         </is>
       </c>
     </row>
@@ -751,10 +794,14 @@
           <t>GM බ්‍රෝ, ඔයා කියනවා නේද දැන් උණ සනීපයි කියලා?</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>GM bro, ඔයා කියනවා නේද දන් උනා සනීපයි කියලා?</t>
+        </is>
+      </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -762,9 +809,9 @@
           <t>Greetings</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
-        <is>
-          <t>Evidence: Abbreviation 'GM' not converted to Sinhala. 'bro' left as Roman instead of 'බ්‍රෝ'. 'dan' output as 'දන්' instead of 'දැන්' — missing 'æ' vowel. 'una' becomes 'උනා' instead of 'උණ'.</t>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: 'bro' is left as Roman text instead of being converted to 'බ්‍රෝ'. 'dan' is output as 'දන්' instead of correct 'දැන්' — the 'æ' vowel (ැ) is missing. 'una' becomes 'උනා' with an extra vowel instead of correct 'උණ' with retroflex 'ණ'.</t>
         </is>
       </c>
     </row>
@@ -789,10 +836,14 @@
           <t>plz මේක ඉක්මනට ඕන</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr"/>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>please මේක ඉක්මනට ඕන</t>
+        </is>
+      </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -800,9 +851,9 @@
           <t>Requests</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>Rationale: The system fails to maintain consistency in word choices when processing a simple request. It replaces the English abbreviation 'plz' with the full Sinhala word 'please' in the actual output, while the expected output requires maintaining the original informal shorthand or character mapping, leading to a character-level mismatch.</t>
+      <c r="H8" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: Abbreviation 'plz' is expanded to full English word 'please' instead of being preserved as 'plz' as required in the expected output — system incorrectly expands the abbreviation rather than keeping the original shorthand form.</t>
         </is>
       </c>
     </row>
@@ -834,7 +885,7 @@
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -842,9 +893,9 @@
           <t>Requests</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr">
-        <is>
-          <t>The system fails to correctly identify and list individual English words when provided as a comma-separated sequence within a Sinhala-focused prompt. Instead of treating 'Mangoes, Bananas, Papayas'' as distinct entities to be maintained, it attempts to phonetically transliterate them, violating the user's intent to provide a clean English list.</t>
+      <c r="H9" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: 'oya' is output as 'ඔය' instead of 'ඔයා' — final long vowel 'ා' dropped. 'kiwapu' becomes 'කිවපු' missing the long vowel. 'Mangoes' is phonetically converted to 'මන්ගෝස්' instead of being preserved as English — system incorrectly transliterates English proper nouns inside a list.</t>
         </is>
       </c>
     </row>
@@ -876,7 +927,7 @@
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -884,9 +935,9 @@
           <t>Responses</t>
         </is>
       </c>
-      <c r="H10" s="3" t="inlineStr">
-        <is>
-          <t>Evidence: Abbreviation 'mm' for 'mama/මම' converted to consonant cluster 'ම්ම්' — vowel dropped producing invalid Sinhala. 'aniwaryen' becomes 'අනිවාර්යෙන්' missing a 'ය' compared to correct 'අනිවාර්යයෙන්'.</t>
+      <c r="H10" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: Abbreviation 'mm' for 'mama/මම' is output as 'ම්ම්' — a consonant cluster without a vowel, producing invalid Sinhala. 'aniwaryen' becomes 'අනිවාර්යෙන්' missing a 'ය' syllable compared to correct 'අනිවාර්යයෙන්'.</t>
         </is>
       </c>
     </row>
@@ -911,10 +962,14 @@
           <t>මෙන්න ඔයා ගන්න කියපු ලිස්ට් එක: 'Books, Pens, Erasers'</t>
         </is>
       </c>
-      <c r="E11" s="3" t="n"/>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>මෙන්න ඔය ගන්ඩ කිවපු ලිස්ට් එක: 'බුක්ස් , පේන්ස් , Erasers '</t>
+        </is>
+      </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -922,9 +977,9 @@
           <t>Responses</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr">
-        <is>
-          <t>Rationale: The system fails to maintain the original English nouns for list items ('Apples, Oranges, Grapes') within a Sinhala response. It phonetically transliterates these items into Sinhala script ('අප්පල්ස්, ග්‍රේප්ස්'), which is unsuitable for professional or clear communication where original English terms are expected to be preserved as per the instruction.</t>
+      <c r="H11" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: 'oya' output as 'ඔය' instead of 'ඔයා' — final vowel dropped. English list items 'Books' and 'Pens' are phonetically converted to 'බුක්ස්' and 'පේන්ස්' instead of being preserved as English words — system incorrectly applies Sinhala phonetics to English nouns in a list context.</t>
         </is>
       </c>
     </row>
@@ -956,7 +1011,7 @@
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -964,9 +1019,9 @@
           <t>Repeated Words</t>
         </is>
       </c>
-      <c r="H12" s="3" t="inlineStr">
-        <is>
-          <t>Evidence: Repeated word 'hadei' output as 'හඩේඉ' instead of 'හැදෙයි' — 'æ' vowel missing and wrong vowel sequence applied to both repeated instances changing the word meaning entirely.</t>
+      <c r="H12" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: Repeated word 'hadei' is output as 'හදේයි' instead of correct 'හැදෙයි' — the 'æ' vowel (ැ) is missing from both instances, changing the meaning of the word. The error applies consistently to both repeated occurrences.</t>
         </is>
       </c>
     </row>
@@ -991,10 +1046,14 @@
           <t>හොඳයි හොඳයි, අපි ඔක්කොම හෙට උදේ එමු</t>
         </is>
       </c>
-      <c r="E13" s="3" t="n"/>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>හොදි හොදි, අපි ඔක්කොම හෙට උදේ එමු</t>
+        </is>
+      </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -1002,9 +1061,9 @@
           <t>Repeated Words</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr">
-        <is>
-          <t>Evidence: Repeated spelling variant 'hodi' output as 'හොදී' instead of correct 'හොඳයි' — missing 'ඳ' character and wrong vowel ending applied to both repeated instances.</t>
+      <c r="H13" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: Repeated spelling variant 'hodi' is output as 'හොදි' instead of correct 'හොඳයි' — the 'ඳ' character is missing and wrong vowel ending applied. The error is consistent across both repeated instances of the word.</t>
         </is>
       </c>
     </row>
@@ -1036,7 +1095,7 @@
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -1044,9 +1103,9 @@
           <t>Inputs with Punctuation Marks</t>
         </is>
       </c>
-      <c r="H14" s="3" t="inlineStr">
-        <is>
-          <t>Evidence: Extended abbreviation 'plzzz' after ellipsis converted to English 'please' instead of being preserved as 'plzzz'. Space before ellipsis also missing in output.</t>
+      <c r="H14" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: Extended abbreviation 'plzzz' after ellipsis is converted to full English word 'please' instead of being preserved as 'plzzz' as required in expected output. Space before '...' is also missing in output.</t>
         </is>
       </c>
     </row>
@@ -1071,10 +1130,14 @@
           <t>Sry, මම තව දවසක් ගන්නවා. හෙට ගෙනත් දෙන්නම්</t>
         </is>
       </c>
-      <c r="E15" s="3" t="n"/>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>ස්රයි, මං තව දවසක් ගන්නවා. හෙට ගෙනත් දෙන්නම්</t>
+        </is>
+      </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -1082,9 +1145,9 @@
           <t>Inputs with Punctuation Marks</t>
         </is>
       </c>
-      <c r="H15" s="3" t="inlineStr">
-        <is>
-          <t>Evidence: 'sry' phonetically converted to 'ස්රයි' instead of being preserved as 'Sry'. 'man' converted to 'මං' instead of 'මම'. Space after comma also dropped. Period at end missing.</t>
+      <c r="H15" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: 'sry' is phonetically converted to 'ස්රයි' instead of being preserved as 'Sry'. 'man' is converted to 'මං' (informal first person) instead of correct 'මම' — different Sinhala pronoun produced from the abbreviated input.</t>
         </is>
       </c>
     </row>
@@ -1109,10 +1172,14 @@
           <t>අනේ මට දැන් සමා වෙන්න ඕනේ. මම ආයේ එහෙම කරන්නේ නෑ</t>
         </is>
       </c>
-      <c r="E16" s="3" t="n"/>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>අනේ මට දැන් සමාව වෙන්න ඕන්නෑ. මං ආයෙ එහෙම කරන්නෙ නෑ</t>
+        </is>
+      </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -1120,9 +1187,9 @@
           <t>Romanization / Spelling Variants</t>
         </is>
       </c>
-      <c r="H16" s="3" t="inlineStr">
-        <is>
-          <t>Evidence: Spelling variant 'onne' converted to 'ඕන්නෑ' (meaning 'not needed') instead of correct 'ඕනේ' — completely reverses sentence meaning. Also 'Samaa wenna' merged incorrectly to 'සමාවෙන්න'.</t>
+      <c r="H16" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: Spelling variant 'onne' is incorrectly converted to 'ඕන්නෑ' (meaning 'not needed/don't want') instead of correct 'ඕනේ' (meaning 'need to') — completely reversing the sentence meaning from positive to negative. 'man' also converted to 'මං' instead of 'මම'.</t>
         </is>
       </c>
     </row>
@@ -1144,13 +1211,17 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>ඔයාට හෙට යුනි යන්න ඕනේ, මතක ඇතුව එන්න</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="n"/>
+          <t>ඔයාට හෙට uni යන්න ඕනේ, මතක ඇතුව එන්න</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>ඔයාට හෙට උනි යන්න ඕන්නෑ, මතක අතුව එන්න</t>
+        </is>
+      </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -1158,9 +1229,9 @@
           <t>Romanization / Spelling Variants</t>
         </is>
       </c>
-      <c r="H17" s="3" t="inlineStr">
-        <is>
-          <t>Evidence: Clipped form 'uni' phonetically converted to 'උනි' instead of 'යුනි'. Comma between clauses dropped. Demonstrates both spelling variant failure and clipped word mishandling.</t>
+      <c r="H17" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: Spelling variant 'onne' again produces wrong negative meaning 'ඕන්නෑ' instead of correct 'ඕනේ'. Clipped word 'uni' is phonetically converted to 'උනි' instead of expected 'uni' — system applies Sinhala phonetics to an English clipped form that should be preserved.</t>
         </is>
       </c>
     </row>
@@ -1182,13 +1253,17 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>මචෝ ඔයා යුනි යද්දී මට කියන්න, මාත් එක්ක එන්නම්</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="n"/>
+          <t>මචෝ ඔයා uni යද්දී මට කියන්න, මාත් එක්ක එන්නම්</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>මචෝ ඔයා උනි යද්දි මට කියන්න, මාත් එක්ක එන්නම්</t>
+        </is>
+      </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -1196,9 +1271,9 @@
           <t>Romanization / Spelling Variants</t>
         </is>
       </c>
-      <c r="H18" s="3" t="inlineStr">
-        <is>
-          <t>Rationale: The system fails to maintain consistency with Sinhala phonetic spelling variants. It transliterates 'uni' into 'උනි' instead of the more standard 'යුනි' or keeping the English shorthand as intended in the expected output, leading to a character mismatch.</t>
+      <c r="H18" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: Clipped word 'uni' is phonetically converted to 'උනි' instead of expected 'uni'. 'yaddi' becomes 'යද්දි' with short vowel instead of correct 'යද්දී' with long vowel — the final long vowel marker is dropped affecting grammatical correctness.</t>
         </is>
       </c>
     </row>
@@ -1223,10 +1298,14 @@
           <t>මචෝ මේ video එක edit-කරලා දෙන්න. ඒක channel එකට upload-කරලා මචං msg එකක් දාන්න</t>
         </is>
       </c>
-      <c r="E19" s="3" t="n"/>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>මචෝ මේ video එක එඩිට් කරලා දෙන්ඩ. ඒක channel එකට upload කරලා මචන් msg එකක් දාන්න</t>
+        </is>
+      </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -1234,9 +1313,9 @@
           <t>Isolated English Word Insertions in Singlish</t>
         </is>
       </c>
-      <c r="H19" s="3" t="inlineStr">
-        <is>
-          <t>Evidence:The system fails to distinguish between English technical terms and Singlish suffixes when they are hyphenated or closely joined (e.g., 'synchronize-karala'). It attempts to transliterate the entire combined string into phonetic Sinhala script, failing to keep the English term 'synchronize' in its original format.</t>
+      <c r="H19" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: English technical term 'edit' in 'edit-karala' is phonetically converted to 'එඩිට්' instead of being preserved as 'edit'. 'mcn' (abbreviation for 'machan') is converted to 'මචන්' instead of correct 'මචෝ' as used in context — system misidentifies the slang abbreviation.</t>
         </is>
       </c>
     </row>
@@ -1261,10 +1340,14 @@
           <t>මචෝ lunch එකට මොනවාද තියෙන්නේ? අපිට fast food order කරන්න පුළුවන්ද?</t>
         </is>
       </c>
-      <c r="E20" s="3" t="n"/>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>මචෝ lunch එකට මොනාද තියෙන්නේ? අපිට fast food order කරන්න පුළුවන්ද?</t>
+        </is>
+      </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -1272,9 +1355,9 @@
           <t>Isolated English Word Insertions in Singlish</t>
         </is>
       </c>
-      <c r="H20" s="3" t="inlineStr">
-        <is>
-          <t>Rationale: The system exhibits inconsistency when handling common English nouns ('lunch', 'order') within a Singlish sentence. Instead of preserving the English script as specified in the expected output, it phonetically transliterates them into Sinhala script, failing the bilingual formatting requirement</t>
+      <c r="H20" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: 'monada' is output as 'මොනාද' instead of correct 'මොනවාද' — a syllable is dropped producing a different Sinhala word. The rest of the sentence including 'fast food' and 'order' is handled correctly, making this a selective vowel-dropping failure.</t>
         </is>
       </c>
     </row>
@@ -1299,10 +1382,14 @@
           <t>මචෝ, ඔයා system එකට log වෙන්න. මම තව පොඩ්ඩක් ගිහින් msg එකක් දාන්න ඕන නේද?</t>
         </is>
       </c>
-      <c r="E21" s="3" t="n"/>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>මචෝ, ඔය system එකට log වෙන්න. මං තව පොඩ්ඩක් ගිහින් msg එකක් දාන්න ඕන නේද?</t>
+        </is>
+      </c>
       <c r="F21" s="6" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -1310,9 +1397,9 @@
           <t>Multi-Word English Phrases in Singlish</t>
         </is>
       </c>
-      <c r="H21" s="3" t="inlineStr">
-        <is>
-          <t>Rationale: The system fails to correctly handle English phrases like 'log wenna'. It phonetically transliterates the English word 'log' into Sinhala ('ලොග්') and changes the context of the sentence, resulting in a mismatch with the expected output that requires specific script preservation for technical actions.</t>
+      <c r="H21" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: 'oya' is output as 'ඔය' instead of correct 'ඔයා' — final long vowel 'ා' dropped. 'man' is converted to 'මං' instead of correct 'මම' — system produces different informal pronoun from the abbreviated input form.</t>
         </is>
       </c>
     </row>
@@ -1337,10 +1424,14 @@
           <t>ඔයාගේ phone එකට මේ App එක දාගන්න. ඒක මාර ලේසි</t>
         </is>
       </c>
-      <c r="E22" s="3" t="n"/>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>ඔයාගෙ phone එකට මේ app එක දාගන්න. ඒක මාර ලේසි</t>
+        </is>
+      </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -1348,9 +1439,9 @@
           <t>Multi-Word English Phrases in Singlish</t>
         </is>
       </c>
-      <c r="H22" s="3" t="inlineStr">
-        <is>
-          <t>Evidence: 'app' phonetically converted to 'අප්ප්' — consonant cluster with hal kirima instead of preserving English word 'App'. Period at end also dropped from output.</t>
+      <c r="H22" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: 'oyage' is output as 'ඔයාගෙ' instead of correct 'ඔයාගේ' — the long vowel ending 'ේ' is replaced by short 'ෙ' changing the possessive form. 'app' is correctly preserved but lowercase instead of required 'App' with capital A.</t>
         </is>
       </c>
     </row>
@@ -1375,10 +1466,14 @@
           <t>පුළුවන් නම් මේ link එක හැමෝම එක්ක share කරන්න. ඒක ගොඩක් වටිනවා</t>
         </is>
       </c>
-      <c r="E23" s="3" t="n"/>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>පුළුවන් නම් මේ link එක හැමෝම එක්ක ශ්ර් කරන්න. ඒක ගොඩක් වටිනවා</t>
+        </is>
+      </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -1386,9 +1481,9 @@
           <t>English Digital Terms in Singlish</t>
         </is>
       </c>
-      <c r="H23" s="3" t="inlineStr">
-        <is>
-          <t>Evidence: Abbreviation 'shr' for 'share' partially converted to 'ශ්‍ර' — only first two characters phonetically rendered, rest dropped, producing meaningless output. Period also missing.</t>
+      <c r="H23" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: Abbreviation 'shr' for 'share' is partially converted to 'ශ්ර්' — only the first consonants are phonetically rendered and the result is an invalid Sinhala consonant cluster. The full word 'share' is not reconstructed and the output is meaningless.</t>
         </is>
       </c>
     </row>
@@ -1413,10 +1508,14 @@
           <t>ඔයා photo එක pc එකේ තියෙනවා. ඒක බලන්න</t>
         </is>
       </c>
-      <c r="E24" s="3" t="n"/>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>ඔය photo එක pc එකේ තියෙනවා. ඒක බලන්න</t>
+        </is>
+      </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -1424,9 +1523,9 @@
           <t>English Digital Terms in Singlish</t>
         </is>
       </c>
-      <c r="H24" s="3" t="inlineStr">
-        <is>
-          <t>Evidence: 'eke' incorrectly output as 'ඒකේ' instead of correct 'එකේ' — wrong vowel applied after platform abbreviation 'IG'. Period at end also missing from output.</t>
+      <c r="H24" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: 'oya' is output as 'ඔය' instead of correct 'ඔයා' — final long vowel 'ා' dropped, changing the pronoun. This is a consistent pattern where 'oya' loses its final vowel in the transliteration output.</t>
         </is>
       </c>
     </row>
@@ -1436,35 +1535,39 @@
           <t>Neg_024</t>
         </is>
       </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>eya heta loku eka ganiwi. eka hondayi</t>
-        </is>
-      </c>
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t>එයා හෙට ලොකු එක ගනීවි. ඒක හොඳයි</t>
-        </is>
-      </c>
-      <c r="E25" s="3" t="n"/>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>oya putput eke aluth adds baluwada?</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>ඔය putput එකේ අලුත් adds බැලුවද?</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>ඔය පුට්පුට් එකේ අලුත් adds බැලුවද?</t>
+        </is>
+      </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G25" s="2" t="inlineStr">
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G25" s="9" t="inlineStr">
         <is>
           <t>Platform/App Names in Singlish</t>
         </is>
       </c>
-      <c r="H25" s="3" t="inlineStr">
-        <is>
-          <t>Evidence: 'eya' output as 'එය' (formal/literary pronoun) instead of colloquial 'එයා'. 'eka' becomes 'ඒක' with wrong vowel instead of 'එක'. Period also dropped.</t>
+      <c r="H25" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: The system fails to maintain the English script for  specific app name ('putput'). Instead of preserving the technical branding in English as required by the expected output, the system phonetically transliterates them into Sinhala script, leading to a loss of brand identity and technical accuracy.</t>
         </is>
       </c>
     </row>
@@ -1481,28 +1584,32 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>karunakarala oyage DOB eka methana danna. eka apita godak wadagath</t>
+          <t>oya Instagram eke aluth reels baluwada?</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>කරුණාකරලා ඔයාගේ DOB එක මෙතන දාන්න. ඒක අපිට ගොඩක් වැදගත්</t>
-        </is>
-      </c>
-      <c r="E26" s="3" t="n"/>
+          <t>ඔයා Instagram එකේ අලුත් reels බැලුවද?</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>ඔයා Instagram එකේ අලුත්‍රීල්ස් බැලුවද?</t>
+        </is>
+      </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>English Abbreviations/Acronyms in Singlish</t>
-        </is>
-      </c>
-      <c r="H26" s="3" t="inlineStr">
-        <is>
-          <t>Evidence: 'eka' following all-caps acronym 'DOB' incorrectly output as 'ඒක' instead of 'එක' — system applies wrong vowel when processing the word immediately after an acronym.</t>
+          <t>Platform/App Names in Singlish</t>
+        </is>
+      </c>
+      <c r="H26" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: The system fails to maintain the English script for  specific feature terms ('reels'). Instead of preserving the technical branding in English as required by the expected output, the system phonetically transliterates them into Sinhala script, leading to a loss of brand identity and technical accuracy.</t>
         </is>
       </c>
     </row>
@@ -1519,18 +1626,22 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>oya aluth sinduwa hondayi. eka bathiya ft santhush karapu ekakda?</t>
+          <t>karunakarala oyage DOB eka methana danna. eka apita godak wadagath</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>ඔයා අලුත් සින්දුව හොඳයි. ඒක භාතිය ft සන්තුෂ් කරපු එකක්ද?</t>
-        </is>
-      </c>
-      <c r="E27" s="3" t="n"/>
+          <t>කරුණාකරලා ඔයාගේ DOB එක මෙතන දාන්න. ඒක අපිට ගොඩක් වැදගත්</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>කරුණාකරලා ඔයාගේ DOB ඒක මෙතන දාන්න. ඒක අපිට ගොඩක් වැදගත්</t>
+        </is>
+      </c>
       <c r="F27" s="6" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -1538,9 +1649,9 @@
           <t>English Abbreviations/Acronyms in Singlish</t>
         </is>
       </c>
-      <c r="H27" s="3" t="inlineStr">
-        <is>
-          <t>Evidence: Abbreviation 'ft' (featuring) phonetically converted to 'ෆෘට්' — system applies Sinhala phonetics to the abbreviation instead of preserving it as 'ft' in the output.</t>
+      <c r="H27" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: 'eka' immediately following all-caps acronym 'DOB' is incorrectly output as 'ඒක' instead of correct 'එක' — system applies wrong vowel when processing a word that immediately follows an uppercase acronym.</t>
         </is>
       </c>
     </row>
@@ -1557,28 +1668,32 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>oya pro version eka use karanna. eke aluth feature ekak thiyenawa</t>
+          <t>oya aluth sinduwa hondayi. eka bathiya ft santhush karapu ekakda?</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>ඔයා pro version එක use කරන්න. එකේ අලුත් feature එකක් තියෙනවා</t>
-        </is>
-      </c>
-      <c r="E28" s="3" t="n"/>
+          <t>ඔයා අලුත් සින්දුව හොඳයි. ඒක භාතිය ft සන්තුෂ් කරපු එකක්ද?</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>ඔය අලුත් සින්දුව හොඳයි. ඒක බතිය ෆෘට් සන්තුෂ් කරපු එකක්ද?</t>
+        </is>
+      </c>
       <c r="F28" s="6" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>English Clipped Forms in Singlish</t>
-        </is>
-      </c>
-      <c r="H28" s="3" t="inlineStr">
-        <is>
-          <t>Evidence: Clipped forms like 'app', 'fb', 'pro' all phonetically converted to Sinhala — system should preserve English technical clipped words rather than applying Sinhala phonetics.</t>
+          <t>English Abbreviations/Acronyms in Singlish</t>
+        </is>
+      </c>
+      <c r="H28" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: Abbreviation 'ft' (featuring) is phonetically converted to 'ෆෘට්' — system applies Sinhala phonetic rules to the abbreviation instead of preserving it as 'ft'. Also 'oya' becomes 'ඔය' instead of 'ඔයා' and 'bathiya' becomes 'බතිය' instead of 'භාතිය'.</t>
         </is>
       </c>
     </row>
@@ -1595,18 +1710,22 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>ada uni yanna bari wenawa. lab eke wadak thiyenawa</t>
+          <t>oya pro version eka use karanna. eke aluth feature ekak thiyenawa</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>අද Uni යන්න බැරි වෙනවා. Lab එකේ වැඩක් තියෙනවා</t>
-        </is>
-      </c>
-      <c r="E29" s="3" t="n"/>
+          <t>ඔයා pro version එක use කරන්න. එකේ අලුත් feature එකක් තියෙනවා</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>ඔයා ප්රෝ version එක use කරන්න. ඒකේ අලුත් feature එකක් තියෙනවා</t>
+        </is>
+      </c>
       <c r="F29" s="6" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -1614,9 +1733,9 @@
           <t>English Clipped Forms in Singlish</t>
         </is>
       </c>
-      <c r="H29" s="3" t="inlineStr">
-        <is>
-          <t>Evidence: Clipped word 'uni' phonetically converted to 'උනි' instead of correct 'යුනි'. 'lab' not capitalized. Period at end missing. System fails to handle clipped English educational terms.</t>
+      <c r="H29" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: Clipped English word 'pro' is phonetically converted to 'ප්රෝ' instead of being preserved as 'pro'. 'eke' following 'pro version' becomes 'ඒකේ' instead of correct 'එකේ' — wrong vowel applied after the clipped form.</t>
         </is>
       </c>
     </row>
@@ -1633,28 +1752,32 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>oyata dan KoHoMaDa? ada wadakata yanne nadda?</t>
+          <t>ada uni yanna bari wenawa. lab eke wadak thiyenawa</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>ඔයාට දැන් කොහොමද? අද වැඩකට යන්නේ නැද්ද?</t>
-        </is>
-      </c>
-      <c r="E30" s="3" t="n"/>
+          <t>අද Uni යන්න බැරි වෙනවා. Lab එකේ වැඩක් තියෙනවා</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>අද උනි යන්න බරි වෙනවා. ලබ් එකේ වැඩක් තියෙනවා</t>
+        </is>
+      </c>
       <c r="F30" s="6" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Place Names Embedded in Singlish</t>
-        </is>
-      </c>
-      <c r="H30" s="3" t="inlineStr">
-        <is>
-          <t>Evidence: CamelCase 'KoHoMaDa' converted to 'කොහොමත්' (meaning 'somehow/anyway') instead of correct 'කොහොමද' — final 'Da' misread producing a completely different Sinhala word.</t>
+          <t>English Clipped Forms in Singlish</t>
+        </is>
+      </c>
+      <c r="H30" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: Clipped word 'uni' is phonetically converted to 'උනි' instead of correct 'Uni'. 'lab' is phonetically converted to 'ලබ්' instead of being preserved as 'Lab'. 'bari' becomes 'බරි' missing the 'æ' vowel — should be 'බැරි'.</t>
         </is>
       </c>
     </row>
@@ -1669,20 +1792,24 @@
           <t>S</t>
         </is>
       </c>
-      <c r="C31" s="7" t="inlineStr">
-        <is>
-          <t>oya heta Weligama yanawada? nathnam Galle wala nawathinawada?</t>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>oyata dan KoHoMaDa? ada wadakata yanne nadda?</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>ඔයා හෙට Weligama යනවාද? නැත්නම් Galle වල නවතිනවාද?</t>
-        </is>
-      </c>
-      <c r="E31" s="3" t="n"/>
+          <t>ඔයාට දැන් කොහොමද? අද වැඩකට යන්නේ නැද්ද?</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>ඔයාට දැන් කොහොමත්ද? අද වදකට යන්නේ නැද්ද?</t>
+        </is>
+      </c>
       <c r="F31" s="6" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -1690,9 +1817,9 @@
           <t>Place Names Embedded in Singlish</t>
         </is>
       </c>
-      <c r="H31" s="3" t="inlineStr">
-        <is>
-          <t>Rationale: The system fails to maintain the original English proper nouns for place names within a Singlish sentence. It attempts to phonetically transliterate these names into Sinhala script, which results in a character mismatch against the expected output that requires preserving the English terminology.</t>
+      <c r="H31" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: CamelCase input 'KoHoMaDa' is converted to 'කොහොමත්ද' instead of correct 'කොහොමද' — the mixed capitalisation causes the system to misread the final 'Da' syllable, producing a word meaning 'somehow' instead of 'how'. 'wadakata' also becomes 'වදකට' losing the long vowel.</t>
         </is>
       </c>
     </row>
@@ -1707,30 +1834,34 @@
           <t>S</t>
         </is>
       </c>
-      <c r="C32" s="3" t="inlineStr">
-        <is>
-          <t>oya Nethmi ekka heta yanna. eka hondai</t>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>oya heta Weligama yanawada? nathnam Galle wala nawathinawada?</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>ඔයා හංසනී කියලා කවුරුවත් දන්නේ නෑ. ඒක හින්දා යන්න</t>
-        </is>
-      </c>
-      <c r="E32" s="3" t="n"/>
+          <t>ඔයා හෙට Weligama යනවාද? නැත්නම් Galle වල නවතිනවාද?</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>ඔයා හෙට වෙලිගම යනවද? නැත්නම් ගාල්ලේ වල නවතිනවද?</t>
+        </is>
+      </c>
       <c r="F32" s="6" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Person Names Embedded in Singlish</t>
-        </is>
-      </c>
-      <c r="H32" s="3" t="inlineStr">
-        <is>
-          <t>Evidence:Person name 'Hansani' not converted to Sinhala script 'හංසනී' — Roman text preserved. Reporting particle 'kiyala/කියලා' also dropped from output changing the sentence structure.</t>
+          <t>Place Names Embedded in Singlish</t>
+        </is>
+      </c>
+      <c r="H32" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: Place name 'Weligama' is phonetically converted to 'වෙලිගම' and 'Galle' to 'ගාල්ලේ' instead of being preserved in their original English romanized form as required in the expected output — system transliterates proper place names.</t>
         </is>
       </c>
     </row>
@@ -1747,18 +1878,22 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Nethmi kohomada, Imasha ennawada?</t>
+          <t>oya Nethmi ekka heta yanna. eka hondai</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>ඔයා නෙත්මි එක්ක හෙට යන්න. ඒක හොඳයි</t>
-        </is>
-      </c>
-      <c r="E33" s="3" t="n"/>
+          <t>ඔයා  නෙත්මි එක්ක හෙට යන්න. ඒක හොඳයි</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>ඔයා නැත්මි එක්ක හෙට යන්න. ඒක හොඳයි</t>
+        </is>
+      </c>
       <c r="F33" s="6" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -1766,9 +1901,9 @@
           <t>Person Names Embedded in Singlish</t>
         </is>
       </c>
-      <c r="H33" s="3" t="inlineStr">
-        <is>
-          <t>Evidence: Person name 'Nethmi' converted to 'නැත්නම්' (meaning 'otherwise/if not') — system misidentifies proper name as Sinhala conditional conjunction, completely changing sentence meaning</t>
+      <c r="H33" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: Person name 'Nethmi' is converted to 'නැත්මි' instead of correct 'නෙත්මි' — the 'e' vowel is changed to 'æ' producing a different and incorrect Sinhala name. The system misidentifies the phonetic mapping of the name.</t>
         </is>
       </c>
     </row>
@@ -1785,28 +1920,32 @@
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>mm me 1st yr eke wadak karanawa. eka thama iwara na</t>
+          <t>Nethmi kohomada, Imasha ennawada?</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>මම මේ 1st yr එකේ වැඩක් කරනවා. ඒක තාම ඉවර නෑ</t>
-        </is>
-      </c>
-      <c r="E34" s="3" t="n"/>
+          <t>ඔයා නෙත්මි එක්ක හෙට යන්න. ඒක හොඳයි</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>නැත්නම් කොහොමද, ඉමාෂා එන්නවද?</t>
+        </is>
+      </c>
       <c r="F34" s="6" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Inputs with Numbers and Numeric Suffixes</t>
-        </is>
-      </c>
-      <c r="H34" s="3" t="inlineStr">
-        <is>
-          <t>Evidence: Abbreviation 'mm' converted to 'මන්' instead of correct 'මම' — wrong pronoun produced. Also 'yr' expanded to full 'year' instead of being preserved as abbreviated form 'yr'.</t>
+          <t>Person Names Embedded in Singlish</t>
+        </is>
+      </c>
+      <c r="H34" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: Person name 'Nethmi' is converted to 'නැත්නම්' (meaning 'otherwise/if not') instead of correct 'නෙත්මි' — system completely misidentifies the proper name as a Sinhala conditional conjunction, changing the sentence meaning entirely.</t>
         </is>
       </c>
     </row>
@@ -1823,18 +1962,22 @@
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>daa oya methana hitiya. eka mataka nadda?</t>
+          <t>mm me 1st yr eke wadak karanawa. eka thama iwara na</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>එදා ඔයා මෙතන හිටියා. ඒක මතක නැද්ද?</t>
-        </is>
-      </c>
-      <c r="E35" s="3" t="n"/>
+          <t>මම මේ 1st yr එකේ වැඩක් කරනවා. ඒක තාම ඉවර නෑ</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>ම්ම් මේ 1st year එකේ වැඩක් කරනවා. ඒක තාම ඉවර නෑ</t>
+        </is>
+      </c>
       <c r="F35" s="6" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -1842,9 +1985,9 @@
           <t>Inputs with Numbers and Numeric Suffixes</t>
         </is>
       </c>
-      <c r="H35" s="3" t="inlineStr">
-        <is>
-          <t>Evidence: 'daa' output as 'දෑ' (meaning 'eyes/things') instead of correct emphatic particle 'එදා' — wrong vowel and missing initial syllable. Word order also differs from expected output.</t>
+      <c r="H35" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: Abbreviation 'mm' is output as 'ම්ම්' — consonant cluster without vowel — instead of correct 'මම'. 'yr' is expanded to full 'year' instead of being preserved as abbreviated 'yr' as required in the expected output.</t>
         </is>
       </c>
     </row>
@@ -1859,30 +2002,34 @@
           <t>S</t>
         </is>
       </c>
-      <c r="C36" s="7" t="inlineStr">
-        <is>
-          <t>oya badu tika LKR6000-kata ganna puluwan. eka godak aduyi</t>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>oya 1 st place gaththa neda? ethakota 78k hambuna neda</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>ඔයා බඩු ටික LKR 6000 කට ගන්න පුළුවන්. ඒක ගොඩක් අඩුයි</t>
-        </is>
-      </c>
-      <c r="E36" s="3" t="n"/>
+          <t>ඔයා 1 st ස්ටේජ් ගත්තා නේද? එතකොට 78k හම්බුණා නේද</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>ඔයා 1 ස්ට් ස්ටේජ් ගත්තා නේද? එතකොට 78ක් හම්බුණා නේද</t>
+        </is>
+      </c>
       <c r="F36" s="6" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Inputs with Currency</t>
-        </is>
-      </c>
-      <c r="H36" s="3" t="inlineStr">
-        <is>
-          <t>Rationale: The system fails to correctly handle currency codes ('LKR', 'USD') when they are concatenated directly with numbers and Singlish suffixes (e.g., 'LKR5000-kata'). It treats the entire string as a single transliteration unit and converts it into phonetic Sinhala script instead of maintaining the standard English currency format, leading to a logical failure.</t>
+          <t>Inputs with Numbers and Numeric Suffixes</t>
+        </is>
+      </c>
+      <c r="H36" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: The system fails to handle alphanumeric combinations and numeric suffixes (e.g., '1st', '78k'). It phonetically transliterates the suffixes into Sinhala script ('ස්ට්', 'කේ') instead of preserving the original English alphanumeric format as required for technical accuracy.</t>
         </is>
       </c>
     </row>
@@ -1897,20 +2044,24 @@
           <t>S</t>
         </is>
       </c>
-      <c r="C37" s="3" t="inlineStr">
-        <is>
-          <t>dollar rate eka kiyada? eka rupees 300-kata wada wadi wenawada?</t>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>oya badu tika LKR6000-kata ganna puluwan. eka godak aduyi</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>dollar rate එක කීයද? ඒක රුපියල් 300 කට වඩා වැඩි වෙනවාද?</t>
-        </is>
-      </c>
-      <c r="E37" s="3" t="n"/>
+          <t>ඔයා බඩු ටික LKR 6000 කට ගන්න. ඒක ගොඩක් අඩුයි</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>ඔය බඩු ටික LKR6000 කට ගන්න පුළුවන්. ඒක ගොඩක් අඩුයි</t>
+        </is>
+      </c>
       <c r="F37" s="6" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -1918,9 +2069,9 @@
           <t>Inputs with Currency</t>
         </is>
       </c>
-      <c r="H37" s="3" t="inlineStr">
-        <is>
-          <t>Evidence: 'rate' phonetically converted to 'රටේ' (meaning 'of the country') — completely wrong word changing question meaning. 'rupees' becomes 'රූපීස්' with wrong long vowel instead of correct 'රුපියල්'.</t>
+      <c r="H37" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: 'LKR6000-kata' is output as 'LKR6000 කට' — hyphen and suffix handled partially correctly but 'puluwan' at end is dropped from output. 'oya' becomes 'ඔය' instead of 'ඔයා' — final vowel dropped, changing the pronoun.</t>
         </is>
       </c>
     </row>
@@ -1935,30 +2086,34 @@
           <t>S</t>
         </is>
       </c>
-      <c r="C38" s="7" t="inlineStr">
-        <is>
-          <t>oya heta 8AM වෙද්දී එන්න. eka godak wadagath</t>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>dollar rate eka kiyada? eka rupees 300-kata wada wadi wenawada?</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>ඔයා හෙට 8AM වෙද්දී එන්න. ඒක ගොඩක් වැදගත්</t>
-        </is>
-      </c>
-      <c r="E38" s="3" t="n"/>
+          <t>dollar rate එක කීයද? ඒක රුපියල් 300 කට වඩා වැඩි වෙනවාද?</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>dollar rate එක කීයද? ඒක rupees 300-කට වඩා වාඩි වෙනවද?</t>
+        </is>
+      </c>
       <c r="F38" s="6" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Inputs with Time Formats</t>
-        </is>
-      </c>
-      <c r="H38" s="3" t="inlineStr">
-        <is>
-          <t>Rationale: The system fails to maintain the original English alphanumeric time format (8AM). It phonetically transliterates the term into Sinhala characters ('8ඒඑම්' or similar), causing a mismatch with the expected English script representation.</t>
+          <t>Inputs with Currency</t>
+        </is>
+      </c>
+      <c r="H38" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: 'rupees' is phonetically converted to 'rupees' preserved in Roman text instead of correct Sinhala 'රුපියල්'. '300-kata' becomes '300-කට' — the hyphen is preserved but the suffix handling differs from expected '300 කට' with a space. 'wadi' becomes 'වාඩි' with wrong long vowel instead of 'වැඩි'.</t>
         </is>
       </c>
     </row>
@@ -1970,23 +2125,27 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>me video eka 5.30 min thiyenawa. eka edit karala ewanna</t>
-        </is>
-      </c>
-      <c r="D39" s="3" t="inlineStr">
-        <is>
-          <t>මේ video එක 5.30 min තියෙනවා. ඒක edit කරලා එවන්න</t>
-        </is>
-      </c>
-      <c r="E39" s="3" t="n"/>
+          <t>oy heta 8 AM weddi enn. eka godak wadagath</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>ඔය හෙට 8 AM වෙද්දී එන්න. ඒක ගොඩක් වැදගත්</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>ඔය හෙට 8 AM වෙද්දි එන්න. ඒක ගොඩක් වැදගත්</t>
+        </is>
+      </c>
       <c r="F39" s="6" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -1994,9 +2153,9 @@
           <t>Inputs with Time Formats</t>
         </is>
       </c>
-      <c r="H39" s="3" t="inlineStr">
-        <is>
-          <t>Rationale: The system incorrectly processes the time-related measurement '5.30 min'. It attempts to transliterate 'min' into a phonetic Sinhala abbreviation ('මිනි' or 'මිනු') instead of preserving the standard English short form, leading to a failure in technical accuracy.</t>
+      <c r="H39" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: 'oy' is output as 'ඔය්' with an incorrect hal kirima instead of correct 'ඔය'. 'weddi' becomes 'වෙද්දි' with short vowel instead of correct 'වෙද්දී' with long vowel — the long vowel marker is dropped, affecting grammatical accuracy.</t>
         </is>
       </c>
     </row>
@@ -2008,33 +2167,37 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>oya 10th May enna puluwanda? eka apita godak hondayi</t>
+          <t>me video eka 5.30 min thiyenawa. eka edit karala ewanna</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>ඔයා 10th May එන්න පුළුවන්ද? ඒක අපිට ගොඩක් හොඳයි</t>
-        </is>
-      </c>
-      <c r="E40" s="3" t="n"/>
+          <t>මේ video එක 5.30 min තියෙනවා. ඒක edit කරලා එවන්න</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>මේ video එක 5.30 මින් තියෙනවා. ඒක එඩිට් කරලා එවන්න</t>
+        </is>
+      </c>
       <c r="F40" s="6" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Inputs with Dates</t>
-        </is>
-      </c>
-      <c r="H40" s="3" t="inlineStr">
-        <is>
-          <t>Rationale: The system fails when English ordinal suffixes ('th') and month names ('May') are used within a Singlish sentence. It phonetically transliterates 'th' into 'ත්' and 'May' into 'මැයි', which deviates from the expected output that requires preserving the English date format.</t>
+          <t>Inputs with Time Formats</t>
+        </is>
+      </c>
+      <c r="H40" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: 'min' is phonetically converted to 'මින්' instead of being preserved as 'min'. 'edit' is converted to 'එඩිට්' instead of being preserved as 'edit' — system incorrectly applies Sinhala phonetics to standard English abbreviations and technical words.</t>
         </is>
       </c>
     </row>
@@ -2046,23 +2209,27 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>oya 12.12 enne nadda? eka loku reduction sale ekak thiyena dawasak</t>
+          <t>oya 10 th May enna puluwanda? eka apita godak hondayi</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>oya 12.12 enne nadda? eka loku reduction sale ekak thiyena dawasak</t>
-        </is>
-      </c>
-      <c r="E41" s="3" t="n"/>
+          <t>ඔයා 10 th May එන්න පුළුවන්ද? ඒක අපිට ගොඩක් හොඳයි</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>ඔයා 10 ත් මැයි එන්න පුළුවන්ද? ඒක අපිට ගොඩක් හොඳයි</t>
+        </is>
+      </c>
       <c r="F41" s="6" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -2070,9 +2237,9 @@
           <t>Inputs with Dates</t>
         </is>
       </c>
-      <c r="H41" s="3" t="inlineStr">
-        <is>
-          <t>Rationale: The system fails to recognize numerical date strings like '12.12' as a specific date or event name. It treats the dots and numbers as a general transliteration task, often leading to formatting errors or incorrect character mapping in the Sinhala output.</t>
+      <c r="H41" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: Ordinal suffix 'th' in '10 th' is converted to 'ත්' (Sinhala consonant cluster) instead of being preserved as 'th'. Month name 'May' is converted to 'මැයි' instead of being preserved as 'May' — system phonetically transliterates English date components.</t>
         </is>
       </c>
     </row>
@@ -2089,28 +2256,32 @@
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>oya 100km-h wada speed yanna epa. eka godak dangerous</t>
-        </is>
-      </c>
-      <c r="D42" s="3" t="inlineStr">
-        <is>
-          <t>ඔයා 100km-h වඩා speed යන්න එපා. ඒක ගොඩක් dangerous</t>
-        </is>
-      </c>
-      <c r="E42" s="3" t="n"/>
+          <t>hi oya 12.12 sale ekata enne nadda? eka loku reduction sale ekak thiyena dawasak</t>
+        </is>
+      </c>
+      <c r="D42" s="7" t="inlineStr">
+        <is>
+          <t>hi ඔය 12.12 sale එකට එන්නෙ නඩ්ඩ? එක ලොකු රෙඩුcටිඔන් සලෙ එකක් තියෙන ඩwඅසක්</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>හි ඔය 12.12 සාලේ එකට එන්නේ නැද්ද? ඒක ලොකු reduction sale එකක් තියෙන දවසක්</t>
+        </is>
+      </c>
       <c r="F42" s="6" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Inputs with Unit of Measurements</t>
-        </is>
-      </c>
-      <c r="H42" s="3" t="inlineStr">
-        <is>
-          <t>Rationale: The system fails to handle combined unit expressions like '100km-h' and 'per-hr'. Instead of maintaining the international standard units in English, it transliterates them into phonetic Sinhala, making the technical measurement unreadable and incorrect.</t>
+          <t>Inputs with Dates</t>
+        </is>
+      </c>
+      <c r="H42" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: 'hi' is converted to 'හි' (Sinhala locative particle) instead of being preserved as 'hi'. The expected output itself contains errors showing the system also fails to correctly transliterate 'reduction' and 'sale' — producing garbled phonetic Sinhala for English promotional terms.</t>
         </is>
       </c>
     </row>
@@ -2127,18 +2298,22 @@
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>oya 10kg-kata wada ganna epa. eka bara wadiyi</t>
+          <t>oya 100km-h wada speed yanna epa. eka godak dangerous</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>ඔයා 10kg කට වඩා ගන්න එපා. ඒක බර වැඩියි</t>
-        </is>
-      </c>
-      <c r="E43" s="3" t="n"/>
+          <t>ඔයා 100km-h වඩා speed යන්න එපා. ඒක ගොඩක් dangerous</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>ඔයා 100km-හ් වඩා speed යන්න එපා. ඒක ගොඩක් dangerous</t>
+        </is>
+      </c>
       <c r="F43" s="6" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -2146,9 +2321,9 @@
           <t>Inputs with Unit of Measurements</t>
         </is>
       </c>
-      <c r="H43" s="3" t="inlineStr">
-        <is>
-          <t>Rationale:The system fails to isolate international standard units (e.g., 'kg') when they are concatenated with numerical values and Singlish suffixes like '-kata'. Instead of preserving the unit in its original English abbreviated form to maintain technical accuracy, the system treats the entire string as a phonological unit and transliterates it into Sinhala script. This results in a character mismatch against the expected output, which requires the English unit to be preserved for automated validation and clarity..</t>
+      <c r="H43" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: Unit expression '100km-h' is converted to '100km-හ්' — the 'h' at end is phonetically converted to 'හ්' (Sinhala consonant) instead of being preserved as part of the speed unit 'km/h'. System incorrectly applies Sinhala phonetics to international measurement unit abbreviations.</t>
         </is>
       </c>
     </row>
@@ -2160,33 +2335,37 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="C44" s="3" t="inlineStr">
-        <is>
-          <t>oya pole badu thama labai. eka hinda heta yanna</t>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>20g-bara athi okanam</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>ඔයා පොළේ බඩු තාම ලාභයි. ඒක හින්දා හෙට යන්න</t>
-        </is>
-      </c>
-      <c r="E44" s="3" t="n"/>
+          <t>20g-බර අති ඕකනම්</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>20gබර ඇති ඕකනම්</t>
+        </is>
+      </c>
       <c r="F44" s="6" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Inputs with Slang and Casual Phrasing</t>
-        </is>
-      </c>
-      <c r="H44" s="3" t="inlineStr">
-        <is>
-          <t>Evidence: Slang word 'labai' (affordable/cheap) incorrectly converted to 'ලයික්' (meaning 'like') — completely wrong word, changing question meaning entirely. 'pole' also missing the retroflex 'ළ'.</t>
+          <t>Inputs with Unit of Measurements</t>
+        </is>
+      </c>
+      <c r="H44" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: Unit 'g' in '20g-bara' is converted to 'ග්' (Sinhala consonant) instead of being preserved as 'g'. 'oknam' is output as 'ඔකනම්' instead of correct 'ඕකනම්' — wrong short vowel used instead of long vowel 'ෝ'.</t>
         </is>
       </c>
     </row>
@@ -2203,18 +2382,22 @@
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>oya pole mal godak labai. eka hinda ganna</t>
+          <t>oya pole badu thama labai. eka hinda heta yanna</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>ඔයා පොළේ මල් ගොඩක් ලාභයි. ඒක හින්දා ගන්න</t>
-        </is>
-      </c>
-      <c r="E45" s="3" t="n"/>
+          <t>ඔයා පොළේ බඩු තාම ලාභයි. ඒක හින්දා හෙට යන්න</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>ඔය පොලේ බඩු තමා ලයි. ඒක හින්දා හෙට යන්න</t>
+        </is>
+      </c>
       <c r="F45" s="6" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -2222,9 +2405,9 @@
           <t>Inputs with Slang and Casual Phrasing</t>
         </is>
       </c>
-      <c r="H45" s="3" t="inlineStr">
-        <is>
-          <t>Evidence: Slang word 'labai' (affordable/cheap) incorrectly converted to 'ලයික්' (meaning 'like') — completely wrong word, changing question meaning entirely. 'pole' also missing the retroflex 'ළ'</t>
+      <c r="H45" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: Slang word 'labai' (meaning affordable/cheap) is incorrectly converted to 'ලයි' — missing 'බ' character producing a meaningless truncated word. 'oya' becomes 'ඔය' instead of correct 'ඔයා' — final long vowel dropped. 'thama' becomes 'තමා' instead of correct 'තාම'.</t>
         </is>
       </c>
     </row>
@@ -2241,28 +2424,32 @@
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>oya nethmi@gmail.com ekata mail ekak danna. nathnam umesha@yahoo.com ekata danna</t>
+          <t>oya pole mal godak labai. eka hinda ganna</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>ඔයා nethmi@gmail.com එකට mail එකක් දාන්න. නැත්නම් umesha@yahoo.com එකට දාන්න</t>
-        </is>
-      </c>
-      <c r="E46" s="3" t="n"/>
+          <t>ඔයා පොළේ මල් ගොඩක් ලාභයි. ඒක හින්දා ගන්න</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>ඔය පොලේ මල් ගොඩක් ලයි. ඒක හින්දා ගන්න</t>
+        </is>
+      </c>
       <c r="F46" s="6" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Online Identifiers in Singlish</t>
-        </is>
-      </c>
-      <c r="H46" s="3" t="inlineStr">
-        <is>
-          <t>Evidence:Username part 'nethmi' or 'umesha' in email address phonetically converted to Sinhala — system incorrectly applies transliteration inside email address, making it invalid.</t>
+          <t>Inputs with Slang and Casual Phrasing</t>
+        </is>
+      </c>
+      <c r="H46" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: Slang word 'labai' (meaning affordable/cheap) is again incorrectly converted to 'ලයි' — 'බ' character dropped producing meaningless output. 'oya' becomes 'ඔය' instead of correct 'ඔයා' — same consistent pattern of final vowel being dropped.</t>
         </is>
       </c>
     </row>
@@ -2279,18 +2466,22 @@
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>oya heta match ekata #LPL_T20_Finals kiyala hashtag ekak danna. eka trend wei</t>
+          <t>oya nethmi@gmail.com ekata mail ekak danna. nathnam umesha@yahoo.com ekata danna</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>ඔයා හෙට match එකට #LPL_T20_Finals කියලා hashtag එකක් දාන්න. ඒක trend වෙයි</t>
-        </is>
-      </c>
-      <c r="E47" s="3" t="n"/>
+          <t>ඔයා nethmi@gmail.com එකට mail එකක් දාන්න. නැත්නම් umesha@yahoo.com එකට දාන්න</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>ඔයා නෙත්මි@gmail.කොම් එකට mail එකක් දාන්න. නැත්නම් umesha@yahoo.කොම් එකට දාන්න</t>
+        </is>
+      </c>
       <c r="F47" s="6" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -2298,9 +2489,9 @@
           <t>Online Identifiers in Singlish</t>
         </is>
       </c>
-      <c r="H47" s="3" t="inlineStr">
-        <is>
-          <t>Evidence: Hashtag '#LPL_T20_Finals' broken apart and partially converted to Sinhala 'එල්පීඑල් T20 Finals' — '#' symbol removed and underscore (_) replaced by spaces, causing the hashtag to lose its social media identifier function</t>
+      <c r="H47" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: Username 'nethmi' in email address 'nethmi@gmail.com' is phonetically converted to 'නෙත්මි' — system incorrectly applies Sinhala transliteration inside an email address. Domain '.com' also converted to '.කොම්' making the email address completely invalid and undeliverable.</t>
         </is>
       </c>
     </row>
@@ -2317,18 +2508,22 @@
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>oya @umesha__96 account ekata message ekak danna. eka eyage main profile eka</t>
+          <t>oya heta match ekata #LPL_T20_Finals kiyala hashtag ekak danna. eka trend wei</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>ඔයා @umesha__96 account එකට message එකක් දාන්න. ඒක එයාගේ main profile එක</t>
-        </is>
-      </c>
-      <c r="E48" s="3" t="n"/>
+          <t>ඔයා හෙට match එකට #LPL_T20_Finals කියලා hashtag එකක් දාන්න. ඒක trend වෙයි</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>ඔයා හෙට match එකට #LPL_T20_Finals කියලා hashtag එකක් දාන්න. ඒක ට්රෙන්ඩ් වෙයි</t>
+        </is>
+      </c>
       <c r="F48" s="6" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -2336,9 +2531,9 @@
           <t>Online Identifiers in Singlish</t>
         </is>
       </c>
-      <c r="H48" s="3" t="inlineStr">
-        <is>
-          <t>Username '@umesha__96' partially converted — 'umesha' transliterated to 'උමේෂා' and '__96' completely dropped. System incorrectly applies Sinhala phonetics to social media username, truncating it.</t>
+      <c r="H48" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: English word 'trend' is phonetically converted to 'ට්රෙන්ඩ්' instead of being preserved as 'trend'. The hashtag '#LPL_T20_Finals' itself is correctly preserved in this case but the surrounding English word fails — showing inconsistent handling of English words.</t>
         </is>
       </c>
     </row>
@@ -2355,18 +2550,22 @@
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>oya instagram.com/umesha__96 link ekata gihin balanna. eka eyage aluthma profile eka</t>
+          <t>oya @ umesha__96 account ekata message ekak danna. eka eyage main profile eka</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>oya instagram.com/umesha__96 link ekata gihin balanna. eka eyage aluthma profile eka</t>
-        </is>
-      </c>
-      <c r="E49" s="3" t="n"/>
+          <t>ඔයා @umesha__96 account එකට message එකක් දාන්න. ඒක එයාගේ main profile එක</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>ඔයා @ umesha__96 account එකට message එකක් දාන්න. ඒක එයාගේ main profile එක</t>
+        </is>
+      </c>
       <c r="F49" s="6" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -2374,9 +2573,9 @@
           <t>Online Identifiers in Singlish</t>
         </is>
       </c>
-      <c r="H49" s="3" t="inlineStr">
-        <is>
-          <t>Evidence: Username 'umesha__96' in URL path partially converted to Sinhala 'උමේෂා' with '__96' dropped — system incorrectly transliterates and truncates the username inside a URL path making it invalid.</t>
+      <c r="H49" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: '@' symbol and username '@umesha__96' are split with a space — output shows '@ umesha__96' instead of '@umesha__96'. The space inserted between '@' and the username breaks the social media mention format making it non-functional.</t>
         </is>
       </c>
     </row>
@@ -2393,28 +2592,32 @@
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>mata heta enna wenne na 😭 sry. eka hinda oya yanna</t>
+          <t>oya instagram.com/umesha__96 link ekata gihin balanna. eka eyage aluthma profile eka</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>මට හෙට එන්න වෙන්නේ නෑ 😭 sry. ඒක හින්දා ඔයා යන්න</t>
-        </is>
-      </c>
-      <c r="E50" s="3" t="n"/>
+          <t>oya instagram.com/umesha__96 link ekata gihin balanna. eka eyage aluthma profile eka</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>ඔය ඉන්ස්ටග්රම්.com/umesha__96 link එකට ගිහින් බලන්න. ඒක එයාගේ අලුත්ම profile එක</t>
+        </is>
+      </c>
       <c r="F50" s="6" t="inlineStr">
         <is>
-          <t>UI Error</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Inputs Containing Emojis</t>
-        </is>
-      </c>
-      <c r="H50" s="3" t="inlineStr">
-        <is>
-          <t>Evidence: After emoji 😭, abbreviation 'sry' phonetically converted to 'ස්රයි' instead of being preserved as 'sry'. System fails to preserve English abbreviations that appear after emoji characters.</t>
+          <t>Online Identifiers in Singlish</t>
+        </is>
+      </c>
+      <c r="H50" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: 'instagram.com' is partially converted — 'ඉන්ස්ටග්රම්' replaces 'instagram' while '.com/umesha__96' path is preserved. System incorrectly applies phonetic transliteration to the domain name portion of the URL while leaving the path unchanged — inconsistent URL handling.</t>
         </is>
       </c>
     </row>
@@ -2429,30 +2632,76 @@
           <t>S</t>
         </is>
       </c>
-      <c r="C51" s="7" t="inlineStr">
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>mata heta enna wenne na 😭. eka hinda oya yanna. Sry</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>මට හෙට එන්න වෙන්නේ නෑ 😭 sry. ඒක හින්දා ඔයා යන්න</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>මට හෙට එන්න වෙන්නේ නෑ 😭. ඒක හින්දා ඔයා යන්න. ස්රයි</t>
+        </is>
+      </c>
+      <c r="F51" s="6" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>Inputs Containing Emojis</t>
+        </is>
+      </c>
+      <c r="H51" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: Abbreviation 'Sry' appearing after emoji 😭 is phonetically converted to 'ස්රයි' — appearing at end of sentence. System fails to preserve English abbreviations that follow emoji characters, applying incorrect phonetic transliteration instead.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="63" customHeight="1">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>Neg_051</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="C52" s="7" t="inlineStr">
         <is>
           <t>oya 4st 🏆 prize eka gaththa. eka niyamayi</t>
         </is>
       </c>
-      <c r="D51" s="3" t="inlineStr">
+      <c r="D52" s="3" t="inlineStr">
         <is>
           <t>ඔයා 4st 🏆 prize එක ගත්තා. ඒක නියමයි</t>
         </is>
       </c>
-      <c r="E51" s="3" t="n"/>
-      <c r="F51" s="6" t="inlineStr">
-        <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G51" s="2" t="inlineStr">
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>ඔයා 4st  prize එක ගත්තා. ඒක නියමයි</t>
+        </is>
+      </c>
+      <c r="F52" s="6" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
         <is>
           <t>Inputs Containing Emojis</t>
         </is>
       </c>
-      <c r="H51" s="3" t="inlineStr">
-        <is>
-          <t>Rationale: The system fails to correctly handle English ordinal indicators ('st') when they appear alongside emojis in a Singlish sentence. It attempts to phonetically transliterate the suffix 'st' into Sinhala characters ('ස්ට්'), causing a character mismatch with the expected output where the English numeric format and emojis should remain unchanged.</t>
+      <c r="H52" s="8" t="inlineStr">
+        <is>
+          <t>Evidence: Emoji '🏆' is completely dropped from the output — system fails to preserve the emoji character that appears between '4st' and 'prize'. The emoji is simply removed rather than being passed through unchanged as required in the expected output.</t>
         </is>
       </c>
     </row>

</xml_diff>